<commit_message>
added image support in exams
</commit_message>
<xml_diff>
--- a/OnlineExamer.Web/wwwroot/Maturi/xlsx/Geography/География_2019.xlsx
+++ b/OnlineExamer.Web/wwwroot/Maturi/xlsx/Geography/География_2019.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Repositories\Examer\Examer\OnlineExamer.Web\wwwroot\Maturi\xlsx\Geography\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nikolay\Repositories\Examer\Examer\OnlineExamer.Web\wwwroot\Maturi\xlsx\Geography\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CCAC608-FDDD-4733-9B33-CB0C24B4089A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E43FCB-60B9-4506-82D6-25E71B29D2FE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{65C2123F-548F-4F17-9539-F7DEA67DA1A9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{65C2123F-548F-4F17-9539-F7DEA67DA1A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="161">
   <si>
     <t>А) движението на Земята около оста й</t>
   </si>
@@ -506,7 +506,16 @@
     <t>Снимка</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/olympiacloudinary/image/upload/v1584045223/Untitled_tywtbg.png</t>
+    <t>https://res.cloudinary.com/olympiacloudinary/image/upload/v1584082317/Geografiq-1_mrc3ws.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/olympiacloudinary/image/upload/v1584082433/Geografiq-2png_hlrku2.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/olympiacloudinary/image/upload/v1584082528/Geografiq-3_or317k.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/olympiacloudinary/image/upload/v1584082595/Geografiq-4_eu7ksn.png</t>
   </si>
 </sst>
 </file>
@@ -875,21 +884,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD93741-D495-49C6-972F-9B71A0877757}">
   <dimension ref="A1:J31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="159.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="75.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="159.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="75.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="81.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="89" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>142</v>
       </c>
@@ -921,7 +930,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>154</v>
       </c>
@@ -949,11 +958,8 @@
       <c r="I2">
         <v>0</v>
       </c>
-      <c r="J2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>113</v>
       </c>
@@ -982,7 +988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>114</v>
       </c>
@@ -1011,7 +1017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>115</v>
       </c>
@@ -1041,7 +1047,7 @@
       </c>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>116</v>
       </c>
@@ -1070,7 +1076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>117</v>
       </c>
@@ -1099,7 +1105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>118</v>
       </c>
@@ -1128,7 +1134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>119</v>
       </c>
@@ -1157,7 +1163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>120</v>
       </c>
@@ -1186,7 +1192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>121</v>
       </c>
@@ -1215,7 +1221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>122</v>
       </c>
@@ -1244,7 +1250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>123</v>
       </c>
@@ -1272,8 +1278,11 @@
       <c r="I13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J13" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>124</v>
       </c>
@@ -1302,7 +1311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>125</v>
       </c>
@@ -1331,7 +1340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>126</v>
       </c>
@@ -1356,11 +1365,8 @@
       <c r="H16">
         <v>1</v>
       </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>127</v>
       </c>
@@ -1388,8 +1394,11 @@
       <c r="I17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J17" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>128</v>
       </c>
@@ -1417,8 +1426,11 @@
       <c r="I18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J18" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>129</v>
       </c>
@@ -1447,7 +1459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>130</v>
       </c>
@@ -1476,7 +1488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>131</v>
       </c>
@@ -1505,7 +1517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>132</v>
       </c>
@@ -1534,7 +1546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>133</v>
       </c>
@@ -1563,7 +1575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>134</v>
       </c>
@@ -1592,7 +1604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>135</v>
       </c>
@@ -1621,7 +1633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>136</v>
       </c>
@@ -1650,7 +1662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>137</v>
       </c>
@@ -1679,7 +1691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>138</v>
       </c>
@@ -1708,7 +1720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>139</v>
       </c>
@@ -1737,7 +1749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>140</v>
       </c>
@@ -1766,7 +1778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>141</v>
       </c>
@@ -1794,8 +1806,17 @@
       <c r="I31">
         <v>0</v>
       </c>
+      <c r="J31" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J13" r:id="rId1" xr:uid="{79F7BE57-D62B-49B7-A384-5DF3457E7163}"/>
+    <hyperlink ref="J17" r:id="rId2" xr:uid="{1A846E46-4366-419B-B737-C4F7585F4A6C}"/>
+    <hyperlink ref="J18" r:id="rId3" xr:uid="{3CF20F2A-0776-4085-9621-C4AF5F1B7D85}"/>
+    <hyperlink ref="J31" r:id="rId4" xr:uid="{A0DFF9B5-D1EA-42E4-8334-DB6A61063070}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>